<commit_message>
Regenerate own-series starter workbooks (README updated for v1.8 and merged reading)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/search/extraction/own_series/extraction_E1_OWN_starter.xlsx
+++ b/search/extraction/own_series/extraction_E1_OWN_starter.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -649,70 +649,76 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="64" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>• Reports 表的 OWN 行请自己填完整（first_author 可写 Own institutional series，year、institution、study_period、n_children_individual 等照提取说明第 4 节）。year 对本院病例适用什么，由统计分析负责人决定；填你认为合适的值并在 notes 里写明。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+          <t>• Reports 表的 OWN 行请自己填完整（first_author 可写 Own institutional series，year、institution、study_period、n_children_individual 等照提取说明第 4 节）。year 对本院病例只用来推算发表时期：协议 v1.8 已定本院 5 例属于“2015 年及以后”，分析脚本不读 OWN 行的 year，填 2026 即可，不必再商量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>• 本院 5 例不做偏倚风险评价，所以不需要和偏倚风险表合并阅读；正式提取的 269 篇才合并（《提取操作说明》第 1 节第 3 步）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>• 只录不可识别的信息：不写姓名、住院号、出生日期、具体日期。用日期算出的间隔，只写间隔本身（如'症状开始 18 小时后入院，入院 2.5 小时后手术'），把天数换算写进 idx_dur_verbatim 或 notes，不写日历日期。</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>• 病历里没有或看不清的项目，不要凭印象或稿件补：写 NR，并在 notes 里说明。拿不准的写在 notes，留待共识讨论。</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>做完以后</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>• 运行 `python3 -I tools/compare_extraction.py check 你的文件.xlsx`，把格式错误改掉。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>• 运行 `python3 -I tools/compare_extraction.py check 你的文件.xlsx`，把格式错误改掉。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>• 把自己的文件交杨俊保管（提取说明第 2.1 节）；两人都交了以后才运行 `compare`，再讨论分歧、建共识文件。</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>• 共识之后，才把共识的 OWN 行和由稿件预填的草稿对照（`python3 -I tools/compare_extraction.py compare 共识文件.xlsx 草稿.xlsx --out 文件夹`；输出里的 E1 指共识文件，E2 指草稿，草稿的 extractor 列是空的，会有警告），用来发现稿件和病历不一致的地方。</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>没有验证的事</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>• 这份文件没有在 Excel 或 WPS 里打开过；下拉列表和版面实际是否正常没有验证。</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1"/>
     <row r="18" ht="54" customHeight="1"/>
     <row r="19" ht="18" customHeight="1"/>
     <row r="20" ht="18" customHeight="1"/>

</xml_diff>